<commit_message>
fix error in xslx
</commit_message>
<xml_diff>
--- a/resources/test/test.xlsx
+++ b/resources/test/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Universität\Master\Masterarbeit\temp\bias-experiment-cai\resources\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2DF9F1-145C-4F69-8403-EE33E69EAC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F206D1D-B655-468D-A7CE-38EA51181AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="75" yWindow="2790" windowWidth="21810" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,37 +57,37 @@
     <t>resources/test/anordnung_1/scene.jpg</t>
   </si>
   <si>
-    <t>resources/test/anordnung_1/face.jpg</t>
-  </si>
-  <si>
     <t>resources/test/anordnung_2/scene.jpg</t>
   </si>
   <si>
-    <t>resources/test/anordnung_2/face.jpg</t>
-  </si>
-  <si>
     <t>resources/test/anordnung_3/scene.jpg</t>
   </si>
   <si>
-    <t>resources/test/anordnung_3/face.jpg</t>
-  </si>
-  <si>
     <t>resources/test/anordnung_4/scene.jpg</t>
   </si>
   <si>
-    <t>resources/test/anordnung_4/face.jpg</t>
-  </si>
-  <si>
-    <t>resources/test/anordnung_1/item.jpg</t>
-  </si>
-  <si>
-    <t>resources/test/anordnung_2/item.jpg</t>
-  </si>
-  <si>
-    <t>resources/test/anordnung_3/item.jpg</t>
-  </si>
-  <si>
-    <t>resources/test/anordnung_4/item.jpg</t>
+    <t>resources/test/anordnung_1/face.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_2/face.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_3/face.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_4/face.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_1/item.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_2/item.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_3/item.png</t>
+  </si>
+  <si>
+    <t>resources/test/anordnung_4/item.png</t>
   </si>
 </sst>
 </file>
@@ -438,7 +438,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
         <v>17</v>
@@ -452,10 +452,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -469,10 +469,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
         <v>19</v>
@@ -486,7 +486,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>16</v>

</xml_diff>